<commit_message>
This is the latest gantt chart update to my Project Methodology course assignment
</commit_message>
<xml_diff>
--- a/2020-02-02_ProMeth_ca_gantt-chart_Emil-Thorsplass.xlsx
+++ b/2020-02-02_ProMeth_ca_gantt-chart_Emil-Thorsplass.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilthorsplass/Desktop/Frontend 1/Courses:Portfolio:Projects/ProMeth/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25B78550-97DA-BE4C-AB6F-6D82CA5442BD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2B1E68-30D9-984E-85C1-C93E4D354D76}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,9 +40,6 @@
     <t>WEEK 10</t>
   </si>
   <si>
-    <t>Start Date: monday 03.02.2020  |  Project duration: 4 weeks</t>
-  </si>
-  <si>
     <t>M</t>
   </si>
   <si>
@@ -274,9 +271,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  Banner &amp; promotion photography </t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">  </t>
     </r>
@@ -289,9 +283,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  Team meeting 17:00</t>
-  </si>
-  <si>
     <t>Membership &amp; Shopping - 8 days</t>
   </si>
   <si>
@@ -307,12 +298,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  Member/shopping front-end</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Developer meeting 8:30</t>
-  </si>
-  <si>
     <t>ET &amp; VA</t>
   </si>
   <si>
@@ -334,13 +319,7 @@
     <t>Project finalization - 2 days</t>
   </si>
   <si>
-    <t xml:space="preserve">  UX &amp; functionality meeting 8:30</t>
-  </si>
-  <si>
     <t>1.5 hr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Dev. wrap-up &amp; finalization</t>
   </si>
   <si>
     <r>
@@ -395,6 +374,27 @@
   </si>
   <si>
     <t xml:space="preserve">  Hans Knudsen</t>
+  </si>
+  <si>
+    <t>Start Date: monday 03.02.2020  |  Project duration: 5 weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Banner &amp; promotion photography </t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Member/shopping front-end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Developer meeting 8:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   UX &amp; functionality meeting 8:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Dev. wrap-up &amp; finalization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Team meeting 17:00</t>
   </si>
 </sst>
 </file>
@@ -843,6 +843,20 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -852,21 +866,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1098,195 +1098,195 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="71"/>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
-      <c r="M1" s="71"/>
-      <c r="N1" s="71"/>
-      <c r="O1" s="71"/>
-      <c r="P1" s="71"/>
+      <c r="A1" s="65"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
     </row>
     <row r="2" spans="1:39" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="71"/>
-      <c r="B2" s="67" t="s">
+      <c r="A2" s="65"/>
+      <c r="B2" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="70" t="s">
+      <c r="C2" s="74"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="72" t="s">
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="65"/>
+      <c r="L2" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="71"/>
-      <c r="Q2" s="71"/>
-      <c r="R2" s="71"/>
-      <c r="S2" s="73" t="s">
+      <c r="M2" s="65"/>
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="71"/>
-      <c r="U2" s="71"/>
-      <c r="V2" s="71"/>
-      <c r="W2" s="71"/>
-      <c r="X2" s="71"/>
-      <c r="Y2" s="71"/>
-      <c r="Z2" s="76" t="s">
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="65"/>
+      <c r="X2" s="65"/>
+      <c r="Y2" s="65"/>
+      <c r="Z2" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="AA2" s="71"/>
-      <c r="AB2" s="71"/>
-      <c r="AC2" s="71"/>
-      <c r="AD2" s="71"/>
-      <c r="AE2" s="71"/>
-      <c r="AF2" s="71"/>
-      <c r="AG2" s="70" t="s">
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="AH2" s="71"/>
-      <c r="AI2" s="71"/>
-      <c r="AJ2" s="71"/>
-      <c r="AK2" s="71"/>
-      <c r="AL2" s="71"/>
-      <c r="AM2" s="71"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="65"/>
+      <c r="AJ2" s="65"/>
+      <c r="AK2" s="65"/>
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
     </row>
     <row r="3" spans="1:39" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="71"/>
-      <c r="B3" s="74" t="s">
+      <c r="A3" s="65"/>
+      <c r="B3" s="67" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="65"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="71"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="AC3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="AG3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="AH3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="AI3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="AJ3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AK3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="AL3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AM3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:39" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="65"/>
+      <c r="B4" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="AA3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="AB3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="AD3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="AF3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="AG3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="AH3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="AJ3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="AK3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AM3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:39" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="71"/>
-      <c r="B4" s="65" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="66"/>
+      <c r="C4" s="72"/>
       <c r="D4" s="6"/>
       <c r="E4" s="7"/>
       <c r="F4" s="8"/>
@@ -1325,15 +1325,15 @@
       <c r="AM4" s="13"/>
     </row>
     <row r="5" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="71"/>
+      <c r="A5" s="65"/>
       <c r="B5" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>16</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>17</v>
       </c>
       <c r="E5" s="17"/>
       <c r="F5" s="18"/>
@@ -1372,15 +1372,15 @@
       <c r="AM5" s="24"/>
     </row>
     <row r="6" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="71"/>
+      <c r="A6" s="65"/>
       <c r="B6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="D6" s="25" t="s">
         <v>19</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>20</v>
       </c>
       <c r="E6" s="26"/>
       <c r="F6" s="27"/>
@@ -1419,15 +1419,15 @@
       <c r="AM6" s="24"/>
     </row>
     <row r="7" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="71"/>
+      <c r="A7" s="65"/>
       <c r="B7" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="D7" s="25" t="s">
         <v>22</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>23</v>
       </c>
       <c r="F7" s="30"/>
       <c r="G7" s="31"/>
@@ -1465,15 +1465,15 @@
       <c r="AM7" s="24"/>
     </row>
     <row r="8" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="71"/>
+      <c r="A8" s="65"/>
       <c r="B8" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E8" s="18"/>
       <c r="F8" s="18"/>
@@ -1512,15 +1512,15 @@
       <c r="AM8" s="24"/>
     </row>
     <row r="9" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="71"/>
+      <c r="A9" s="65"/>
       <c r="B9" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E9" s="18"/>
       <c r="F9" s="18"/>
@@ -1558,15 +1558,15 @@
       <c r="AM9" s="24"/>
     </row>
     <row r="10" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="71"/>
+      <c r="A10" s="65"/>
       <c r="B10" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="25" t="s">
         <v>26</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="25" t="s">
-        <v>27</v>
       </c>
       <c r="E10" s="18"/>
       <c r="F10" s="18"/>
@@ -1605,11 +1605,11 @@
       <c r="AM10" s="24"/>
     </row>
     <row r="11" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="71"/>
-      <c r="B11" s="65" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="66"/>
+      <c r="A11" s="65"/>
+      <c r="B11" s="71" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="72"/>
       <c r="D11" s="6"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -1648,15 +1648,15 @@
       <c r="AM11" s="13"/>
     </row>
     <row r="12" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="71"/>
+      <c r="A12" s="65"/>
       <c r="B12" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="D12" s="25" t="s">
         <v>30</v>
-      </c>
-      <c r="D12" s="25" t="s">
-        <v>31</v>
       </c>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
@@ -1695,15 +1695,15 @@
       <c r="AM12" s="24"/>
     </row>
     <row r="13" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="71"/>
+      <c r="A13" s="65"/>
       <c r="B13" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="D13" s="25" t="s">
         <v>33</v>
-      </c>
-      <c r="D13" s="25" t="s">
-        <v>34</v>
       </c>
       <c r="E13" s="23"/>
       <c r="F13" s="23"/>
@@ -1742,15 +1742,15 @@
       <c r="AM13" s="24"/>
     </row>
     <row r="14" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="71"/>
+      <c r="A14" s="65"/>
       <c r="B14" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="E14" s="18"/>
       <c r="F14" s="18"/>
@@ -1789,15 +1789,15 @@
       <c r="AM14" s="24"/>
     </row>
     <row r="15" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="71"/>
+      <c r="A15" s="65"/>
       <c r="B15" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="D15" s="25" t="s">
         <v>38</v>
-      </c>
-      <c r="D15" s="25" t="s">
-        <v>39</v>
       </c>
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
@@ -1836,15 +1836,15 @@
       <c r="AM15" s="24"/>
     </row>
     <row r="16" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="71"/>
+      <c r="A16" s="65"/>
       <c r="B16" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="15" t="s">
-        <v>41</v>
-      </c>
       <c r="D16" s="25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E16" s="18"/>
       <c r="F16" s="18"/>
@@ -1883,11 +1883,11 @@
       <c r="AM16" s="24"/>
     </row>
     <row r="17" spans="1:39" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="71"/>
-      <c r="B17" s="65" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="66"/>
+      <c r="A17" s="65"/>
+      <c r="B17" s="71" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="72"/>
       <c r="D17" s="6"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
@@ -1926,15 +1926,15 @@
       <c r="AM17" s="13"/>
     </row>
     <row r="18" spans="1:39" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="71"/>
+      <c r="A18" s="65"/>
       <c r="B18" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" s="43" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E18" s="44"/>
       <c r="F18" s="44"/>
@@ -1973,15 +1973,15 @@
       <c r="AM18" s="24"/>
     </row>
     <row r="19" spans="1:39" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="71"/>
+      <c r="A19" s="65"/>
       <c r="B19" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C19" s="42" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="43" t="s">
         <v>33</v>
-      </c>
-      <c r="D19" s="43" t="s">
-        <v>34</v>
       </c>
       <c r="E19" s="44"/>
       <c r="F19" s="44"/>
@@ -2020,15 +2020,15 @@
       <c r="AM19" s="24"/>
     </row>
     <row r="20" spans="1:39" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="71"/>
+      <c r="A20" s="65"/>
       <c r="B20" s="47" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="C20" s="42" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D20" s="43" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" s="45"/>
       <c r="F20" s="45"/>
@@ -2067,15 +2067,15 @@
       <c r="AM20" s="24"/>
     </row>
     <row r="21" spans="1:39" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="71"/>
+      <c r="A21" s="65"/>
       <c r="B21" s="14" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C21" s="42" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D21" s="43" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E21" s="44"/>
       <c r="F21" s="44"/>
@@ -2114,15 +2114,15 @@
       <c r="AM21" s="24"/>
     </row>
     <row r="22" spans="1:39" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="71"/>
+      <c r="A22" s="65"/>
       <c r="B22" s="48" t="s">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C22" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="25" t="s">
         <v>16</v>
-      </c>
-      <c r="D22" s="25" t="s">
-        <v>17</v>
       </c>
       <c r="E22" s="23"/>
       <c r="F22" s="23"/>
@@ -2161,11 +2161,11 @@
       <c r="AM22" s="24"/>
     </row>
     <row r="23" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="71"/>
-      <c r="B23" s="65" t="s">
-        <v>48</v>
-      </c>
-      <c r="C23" s="66"/>
+      <c r="A23" s="65"/>
+      <c r="B23" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="72"/>
       <c r="D23" s="49"/>
       <c r="E23" s="9"/>
       <c r="F23" s="10"/>
@@ -2204,15 +2204,15 @@
       <c r="AM23" s="13"/>
     </row>
     <row r="24" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="71"/>
+      <c r="A24" s="65"/>
       <c r="B24" s="14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C24" s="42" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="43" t="s">
         <v>38</v>
-      </c>
-      <c r="D24" s="43" t="s">
-        <v>39</v>
       </c>
       <c r="E24" s="44"/>
       <c r="F24" s="44"/>
@@ -2251,15 +2251,15 @@
       <c r="AM24" s="24"/>
     </row>
     <row r="25" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="71"/>
+      <c r="A25" s="65"/>
       <c r="B25" s="47" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="C25" s="42" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25" s="43" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E25" s="45"/>
       <c r="F25" s="45"/>
@@ -2298,15 +2298,15 @@
       <c r="AM25" s="24"/>
     </row>
     <row r="26" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="71"/>
+      <c r="A26" s="65"/>
       <c r="B26" s="47" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="C26" s="42" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D26" s="43" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E26" s="23"/>
       <c r="F26" s="23"/>
@@ -2345,15 +2345,15 @@
       <c r="AM26" s="24"/>
     </row>
     <row r="27" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="71"/>
+      <c r="A27" s="65"/>
       <c r="B27" s="14" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E27" s="22"/>
       <c r="F27" s="22"/>
@@ -2392,11 +2392,11 @@
       <c r="AM27" s="24"/>
     </row>
     <row r="28" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="71"/>
-      <c r="B28" s="65" t="s">
-        <v>55</v>
-      </c>
-      <c r="C28" s="66"/>
+      <c r="A28" s="65"/>
+      <c r="B28" s="71" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="72"/>
       <c r="D28" s="49"/>
       <c r="E28" s="9"/>
       <c r="F28" s="10"/>
@@ -2435,15 +2435,15 @@
       <c r="AM28" s="13"/>
     </row>
     <row r="29" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="71"/>
+      <c r="A29" s="65"/>
       <c r="B29" s="47" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="C29" s="42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D29" s="43" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E29" s="23"/>
       <c r="F29" s="23"/>
@@ -2482,15 +2482,15 @@
       <c r="AM29" s="24"/>
     </row>
     <row r="30" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="71"/>
+      <c r="A30" s="65"/>
       <c r="B30" s="47" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="C30" s="42" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D30" s="43" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E30" s="23"/>
       <c r="F30" s="23"/>
@@ -2529,15 +2529,15 @@
       <c r="AM30" s="24"/>
     </row>
     <row r="31" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="71"/>
+      <c r="A31" s="65"/>
       <c r="B31" s="51" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C31" s="52" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="53" t="s">
         <v>16</v>
-      </c>
-      <c r="D31" s="53" t="s">
-        <v>17</v>
       </c>
       <c r="E31" s="54"/>
       <c r="F31" s="54"/>
@@ -2578,60 +2578,60 @@
     <row r="32" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="33" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="58" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="35" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B35" s="59" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C35" s="60" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="J35" s="26"/>
       <c r="K35" s="61" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B36" s="59" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C36" s="60" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J36" s="62"/>
       <c r="K36" s="63" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B37" s="59" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C37" s="60" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="J37" s="64"/>
       <c r="K37" s="61" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B38" s="59" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C38" s="60" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B39" s="59" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C39" s="60" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -2658,11 +2658,6 @@
     <row r="61" ht="22.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="AG2:AM2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="Z2:AF2"/>
-    <mergeCell ref="S2:Y2"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B17:C17"/>
@@ -2670,6 +2665,11 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="AG2:AM2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="Z2:AF2"/>
+    <mergeCell ref="S2:Y2"/>
     <mergeCell ref="E2:K2"/>
     <mergeCell ref="L2:R2"/>
   </mergeCells>

</xml_diff>